<commit_message>
M8: fictional town name in the anonymised fixture and importer tests
The anonymised golden fixture also replaces the town (Riverbend), and
golden.test.ts and scale.test.ts no longer name it. Counts unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018XhZwgs4tF2kJryLa9b4fB
</commit_message>
<xml_diff>
--- a/packages/importer/fixtures/sample-register-anonymised.xlsx
+++ b/packages/importer/fixtures/sample-register-anonymised.xlsx
@@ -106,7 +106,7 @@
     <t>Kestrel Metals Group/ Kestrel Aluminium/ Plant</t>
   </si>
   <si>
-    <t>India/ West Bengal/ Belur</t>
+    <t>India/ West Bengal/ Riverbend</t>
   </si>
   <si>
     <t>Person Alpha</t>
@@ -1057,7 +1057,7 @@
     <t>Environment Module</t>
   </si>
   <si>
-    <t>Kestrel Aluminium Limited, Belur , Renewal of Consent to Operate under Water (Prevention and Control of Pollution) Act and Air (Prevention and Control of Pollution) Act</t>
+    <t>Kestrel Aluminium Limited, Riverbend , Renewal of Consent to Operate under Water (Prevention and Control of Pollution) Act and Air (Prevention and Control of Pollution) Act</t>
   </si>
   <si>
     <t>Super Critical</t>

</xml_diff>

<commit_message>
M8: replace the real town name left in the anonymised fixture's comments
Three Owner Comments in sample-register-anonymised.xlsx still named a real
town. The anonymiser now maps it to "Kestrelganj" in every cell, the rebuilt
fixture differs from the old one in exactly those 3 cells, and a new test
fails if any banned name appears anywhere in the fixture.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018XhZwgs4tF2kJryLa9b4fB
</commit_message>
<xml_diff>
--- a/packages/importer/fixtures/sample-register-anonymised.xlsx
+++ b/packages/importer/fixtures/sample-register-anonymised.xlsx
@@ -1710,7 +1710,7 @@
     <t>Pay to the Welfare Commissioner, employer's and employees' contribution, half yearly, before 15th July and 15th January every year in Form D.</t>
   </si>
   <si>
-    <t>No TDS deducted for Unionised employees for the month of June 2022. For Mgm employees TDS deposited by Renukoot</t>
+    <t>No TDS deducted for Unionised employees for the month of June 2022. For Mgm employees TDS deposited by Kestrelganj</t>
   </si>
   <si>
     <t>No TDS figure generated for Unionised emp for the month of Jul 2022 and for Mgm emp TDS directly deposited by Central Payroll Team</t>
@@ -1725,7 +1725,7 @@
     <t>We do not store any flammable gas in pressure vessel</t>
   </si>
   <si>
-    <t>No TDS appear for Unionised emp for Mgm emp TDS deposited by Renukoot</t>
+    <t>No TDS appear for Unionised emp for Mgm emp TDS deposited by Kestrelganj</t>
   </si>
   <si>
     <t>Overtime payment with Wages done</t>
@@ -1821,7 +1821,7 @@
     <t>complete</t>
   </si>
   <si>
-    <t xml:space="preserve">No TDS for Unionised emp for Management emp TDS deposited by Renukoot
+    <t xml:space="preserve">No TDS for Unionised emp for Management emp TDS deposited by Kestrelganj
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
M8: replace the real town name left in the anonymised fixture's comments (#109)
Three Owner Comments in sample-register-anonymised.xlsx still named a real
town. The anonymiser now maps it to "Kestrelganj" in every cell, the rebuilt
fixture differs from the old one in exactly those 3 cells, and a new test
fails if any banned name appears anywhere in the fixture.


Claude-Session: https://claude.ai/code/session_018XhZwgs4tF2kJryLa9b4fB

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/importer/fixtures/sample-register-anonymised.xlsx
+++ b/packages/importer/fixtures/sample-register-anonymised.xlsx
@@ -1710,7 +1710,7 @@
     <t>Pay to the Welfare Commissioner, employer's and employees' contribution, half yearly, before 15th July and 15th January every year in Form D.</t>
   </si>
   <si>
-    <t>No TDS deducted for Unionised employees for the month of June 2022. For Mgm employees TDS deposited by Renukoot</t>
+    <t>No TDS deducted for Unionised employees for the month of June 2022. For Mgm employees TDS deposited by Kestrelganj</t>
   </si>
   <si>
     <t>No TDS figure generated for Unionised emp for the month of Jul 2022 and for Mgm emp TDS directly deposited by Central Payroll Team</t>
@@ -1725,7 +1725,7 @@
     <t>We do not store any flammable gas in pressure vessel</t>
   </si>
   <si>
-    <t>No TDS appear for Unionised emp for Mgm emp TDS deposited by Renukoot</t>
+    <t>No TDS appear for Unionised emp for Mgm emp TDS deposited by Kestrelganj</t>
   </si>
   <si>
     <t>Overtime payment with Wages done</t>
@@ -1821,7 +1821,7 @@
     <t>complete</t>
   </si>
   <si>
-    <t xml:space="preserve">No TDS for Unionised emp for Management emp TDS deposited by Renukoot
+    <t xml:space="preserve">No TDS for Unionised emp for Management emp TDS deposited by Kestrelganj
 </t>
   </si>
   <si>

</xml_diff>